<commit_message>
Correction of translation table
</commit_message>
<xml_diff>
--- a/data/translation_table.xlsx
+++ b/data/translation_table.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\perla\Documents\AT\TeamProject\GitHub\TeamProject\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA050D76-F1A4-4209-905C-F6EB73563578}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5373A87-A3CE-464A-9F83-D77E46E15898}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E84D9C67-06AA-45E9-9F3A-D00EAF183968}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -218,9 +218,6 @@
     <t>LWRB</t>
   </si>
   <si>
-    <t>L.M5</t>
-  </si>
-  <si>
     <t>RWRA</t>
   </si>
   <si>
@@ -239,9 +236,6 @@
     <t>R.AnkleLat</t>
   </si>
   <si>
-    <t>R.M5</t>
-  </si>
-  <si>
     <t>R.Hip.Lat</t>
   </si>
   <si>
@@ -249,6 +243,12 @@
   </si>
   <si>
     <t>L.Toe.Lat</t>
+  </si>
+  <si>
+    <t>RM5</t>
+  </si>
+  <si>
+    <t>LM5</t>
   </si>
 </sst>
 </file>
@@ -826,7 +826,7 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B11" s="8"/>
       <c r="C11" s="8"/>
@@ -916,14 +916,14 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E18" s="2"/>
     </row>
@@ -1076,11 +1076,11 @@
         <v>45</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="D27" s="2"/>
       <c r="E27" s="2" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F27" s="1"/>
     </row>
@@ -1141,40 +1141,40 @@
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E32" s="2"/>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" s="6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E33" s="2"/>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" s="6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E34" s="2"/>
     </row>
@@ -1228,7 +1228,7 @@
         <v>39</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
@@ -1275,7 +1275,7 @@
         <v>38</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D40" s="2" t="s">
         <v>38</v>
@@ -1327,11 +1327,11 @@
         <v>47</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D43" s="2"/>
       <c r="E43" s="2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="F43" s="1"/>
     </row>

</xml_diff>

<commit_message>
DB Simonlehner Marker Labels
</commit_message>
<xml_diff>
--- a/data/translation_table.xlsx
+++ b/data/translation_table.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10525"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\perla\Documents\AT\TeamProject\GitHub\TeamProject\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rosesharifi/Documents/GitHub/TeamProject/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F6DF8DA-5566-461E-815C-1A654B0BF8E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B4978D4-200F-AA4E-AD36-03ED784CB9DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="29540" yWindow="-3260" windowWidth="38080" windowHeight="20780" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="210">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="229">
   <si>
     <t>Rajagopal2015_ViconPlugInGait.osim</t>
   </si>
@@ -655,6 +655,63 @@
   </si>
   <si>
     <t>V.Sacral</t>
+  </si>
+  <si>
+    <t>DB Simonlehner</t>
+  </si>
+  <si>
+    <t>LFRA</t>
+  </si>
+  <si>
+    <t>LIAS</t>
+  </si>
+  <si>
+    <t>SACR2</t>
+  </si>
+  <si>
+    <t>LT1/LT2/LT3</t>
+  </si>
+  <si>
+    <t>LS1/LS2/LS3</t>
+  </si>
+  <si>
+    <t>RFRA</t>
+  </si>
+  <si>
+    <t>RIAS</t>
+  </si>
+  <si>
+    <t>SACR3</t>
+  </si>
+  <si>
+    <t>RT1/RT2/RT3</t>
+  </si>
+  <si>
+    <t>RS1/RS2/RS3</t>
+  </si>
+  <si>
+    <t>SACR1</t>
+  </si>
+  <si>
+    <t>LKNM</t>
+  </si>
+  <si>
+    <t>RKNM</t>
+  </si>
+  <si>
+    <t>LANM</t>
+  </si>
+  <si>
+    <t>RANM</t>
+  </si>
+  <si>
+    <t>LTOET</t>
+  </si>
+  <si>
+    <t>RTOET</t>
+  </si>
+  <si>
+    <t>Extra Markers</t>
   </si>
 </sst>
 </file>
@@ -704,7 +761,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -717,8 +774,14 @@
         <bgColor rgb="FFFFFFCC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -741,11 +804,69 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="0" tint="-0.499984740745262"/>
+      </left>
+      <right style="thin">
+        <color theme="0" tint="-0.499984740745262"/>
+      </right>
+      <top style="thin">
+        <color theme="0" tint="-0.499984740745262"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0" tint="-0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color theme="0" tint="-0.499984740745262"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0" tint="-0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color theme="0" tint="-0.499984740745262"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -770,6 +891,21 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -965,22 +1101,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L1043"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:M1043"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="3" width="15.77734375" customWidth="1"/>
-    <col min="4" max="4" width="15.77734375" style="1" customWidth="1"/>
+    <col min="1" max="3" width="15.83203125" customWidth="1"/>
+    <col min="4" max="4" width="15.83203125" style="1" customWidth="1"/>
     <col min="5" max="5" width="27.33203125" customWidth="1"/>
-    <col min="6" max="6" width="15.44140625" customWidth="1"/>
-    <col min="7" max="7" width="3.44140625" customWidth="1"/>
-    <col min="8" max="8" width="1.88671875" customWidth="1"/>
+    <col min="6" max="6" width="15.5" customWidth="1"/>
+    <col min="7" max="7" width="3.5" customWidth="1"/>
+    <col min="8" max="8" width="1.83203125" customWidth="1"/>
     <col min="9" max="9" width="10" customWidth="1"/>
-    <col min="10" max="10" width="9.6640625" customWidth="1"/>
+    <col min="10" max="10" width="8.6640625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="12.6640625" customWidth="1"/>
-    <col min="12" max="12" width="17.109375" customWidth="1"/>
+    <col min="12" max="12" width="17.1640625" customWidth="1"/>
+    <col min="13" max="13" width="13.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="40.200000000000003" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" ht="43" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1011,8 +1148,11 @@
       <c r="L1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M1" s="3" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>9</v>
       </c>
@@ -1034,8 +1174,11 @@
       <c r="K2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M2" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>13</v>
       </c>
@@ -1057,8 +1200,11 @@
       <c r="K3" s="4" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M3" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>17</v>
       </c>
@@ -1077,8 +1223,11 @@
       <c r="J4" s="1" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M4" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>20</v>
       </c>
@@ -1097,8 +1246,11 @@
       <c r="J5" s="1" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M5" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>23</v>
       </c>
@@ -1119,8 +1271,11 @@
       <c r="J6" s="1" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M6" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>27</v>
       </c>
@@ -1137,8 +1292,11 @@
       <c r="J7" s="1" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M7" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>29</v>
       </c>
@@ -1153,8 +1311,11 @@
       <c r="J8" s="1" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M8" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>30</v>
       </c>
@@ -1175,8 +1336,11 @@
       <c r="J9" s="1" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M9" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>34</v>
       </c>
@@ -1197,8 +1361,11 @@
       <c r="J10" s="1" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M10" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>38</v>
       </c>
@@ -1218,8 +1385,11 @@
       <c r="L11" t="s">
         <v>209</v>
       </c>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M11" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>41</v>
       </c>
@@ -1242,8 +1412,11 @@
       <c r="J12" s="1" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M12" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>46</v>
       </c>
@@ -1261,8 +1434,11 @@
       <c r="J13" s="1" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M13" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>50</v>
       </c>
@@ -1283,8 +1459,11 @@
       <c r="J14" s="1" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M14" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
         <v>54</v>
       </c>
@@ -1302,8 +1481,11 @@
       <c r="J15" s="1" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M15" s="1" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
         <v>58</v>
       </c>
@@ -1324,8 +1506,11 @@
       <c r="J16" s="1" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M16" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
         <v>62</v>
       </c>
@@ -1346,8 +1531,11 @@
       <c r="J17" s="1" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M17" s="1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
         <v>66</v>
       </c>
@@ -1368,8 +1556,11 @@
       <c r="J18" s="1" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M18" s="1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
         <v>70</v>
       </c>
@@ -1400,8 +1591,11 @@
       <c r="L19" s="6" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M19" s="12" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A20" s="7" t="s">
         <v>76</v>
       </c>
@@ -1429,8 +1623,11 @@
       <c r="K20" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M20" s="12" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
         <v>82</v>
       </c>
@@ -1458,8 +1655,11 @@
       <c r="L21" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M21" s="12" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
         <v>88</v>
       </c>
@@ -1490,8 +1690,11 @@
       <c r="L22" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M22" s="1" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A23" s="8" t="s">
         <v>95</v>
       </c>
@@ -1519,8 +1722,11 @@
       <c r="L23" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M23" s="12" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
         <v>101</v>
       </c>
@@ -1551,8 +1757,11 @@
       <c r="L24" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M24" s="1" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
         <v>108</v>
       </c>
@@ -1583,8 +1792,11 @@
       <c r="L25" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M25" s="1" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
         <v>114</v>
       </c>
@@ -1607,8 +1819,11 @@
       <c r="J26" s="1" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M26" s="1" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A27" s="8" t="s">
         <v>118</v>
       </c>
@@ -1634,8 +1849,9 @@
       <c r="L27" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M27" s="1"/>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A28" s="8" t="s">
         <v>125</v>
       </c>
@@ -1658,8 +1874,11 @@
       <c r="J28" s="1" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M28" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
         <v>130</v>
       </c>
@@ -1677,8 +1896,11 @@
       <c r="J29" s="1" t="s">
         <v>130</v>
       </c>
-    </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M29" s="1" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
         <v>134</v>
       </c>
@@ -1699,8 +1921,11 @@
       <c r="J30" s="1" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M30" s="1" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
         <v>138</v>
       </c>
@@ -1718,8 +1943,11 @@
       <c r="J31" s="1" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M31" s="12" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
         <v>142</v>
       </c>
@@ -1740,8 +1968,11 @@
       <c r="J32" s="1" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M32" s="1" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="33" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A33" s="8" t="s">
         <v>146</v>
       </c>
@@ -1762,8 +1993,11 @@
       <c r="J33" s="1" t="s">
         <v>146</v>
       </c>
-    </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M33" s="1" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="34" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A34" s="8" t="s">
         <v>150</v>
       </c>
@@ -1784,8 +2018,11 @@
       <c r="J34" s="1" t="s">
         <v>150</v>
       </c>
-    </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M34" s="1" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="35" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
         <v>154</v>
       </c>
@@ -1816,8 +2053,11 @@
       <c r="L35" s="6" t="s">
         <v>159</v>
       </c>
-    </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M35" s="12" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="36" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A36" s="8" t="s">
         <v>160</v>
       </c>
@@ -1845,8 +2085,11 @@
       <c r="K36" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M36" s="12" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="37" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A37" s="8" t="s">
         <v>166</v>
       </c>
@@ -1870,8 +2113,11 @@
       <c r="L37" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M37" s="12" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="38" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A38" s="8" t="s">
         <v>171</v>
       </c>
@@ -1902,8 +2148,11 @@
       <c r="L38" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M38" s="1" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="39" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A39" s="8" t="s">
         <v>178</v>
       </c>
@@ -1931,8 +2180,11 @@
       <c r="L39" t="s">
         <v>183</v>
       </c>
-    </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M39" s="12" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="40" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A40" s="1" t="s">
         <v>184</v>
       </c>
@@ -1963,8 +2215,11 @@
       <c r="L40" t="s">
         <v>190</v>
       </c>
-    </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M40" s="1" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="41" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A41" s="1" t="s">
         <v>191</v>
       </c>
@@ -1995,8 +2250,11 @@
       <c r="L41" t="s">
         <v>196</v>
       </c>
-    </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M41" s="1" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="42" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A42" s="8" t="s">
         <v>197</v>
       </c>
@@ -2019,8 +2277,11 @@
       <c r="J42" s="1" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M42" s="1" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="43" spans="1:13" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A43" s="8" t="s">
         <v>201</v>
       </c>
@@ -2046,8 +2307,9 @@
       <c r="L43" t="s">
         <v>208</v>
       </c>
-    </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M43" s="13"/>
+    </row>
+    <row r="44" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A44" s="10"/>
       <c r="B44" s="11"/>
       <c r="C44" s="11"/>
@@ -2056,8 +2318,11 @@
       <c r="F44" s="11"/>
       <c r="I44" s="11"/>
       <c r="J44" s="11"/>
-    </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M44" s="14" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="45" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A45" s="10"/>
       <c r="B45" s="11"/>
       <c r="C45" s="11"/>
@@ -2065,8 +2330,11 @@
       <c r="F45" s="11"/>
       <c r="I45" s="11"/>
       <c r="J45" s="11"/>
-    </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M45" s="15" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="46" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A46" s="10"/>
       <c r="B46" s="11"/>
       <c r="C46" s="11"/>
@@ -2074,8 +2342,11 @@
       <c r="F46" s="11"/>
       <c r="I46" s="11"/>
       <c r="J46" s="11"/>
-    </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M46" s="15" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="47" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A47" s="10"/>
       <c r="B47" s="11"/>
       <c r="C47" s="11"/>
@@ -2083,8 +2354,11 @@
       <c r="F47" s="11"/>
       <c r="I47" s="11"/>
       <c r="J47" s="11"/>
-    </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M47" s="15" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="48" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A48" s="10"/>
       <c r="B48" s="11"/>
       <c r="C48" s="11"/>
@@ -2092,8 +2366,11 @@
       <c r="F48" s="11"/>
       <c r="I48" s="11"/>
       <c r="J48" s="11"/>
-    </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="M48" s="15" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="49" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A49" s="10"/>
       <c r="B49" s="11"/>
       <c r="C49" s="11"/>
@@ -2101,8 +2378,11 @@
       <c r="F49" s="11"/>
       <c r="I49" s="11"/>
       <c r="J49" s="11"/>
-    </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="M49" s="15" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="50" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A50" s="10"/>
       <c r="B50" s="11"/>
       <c r="C50" s="11"/>
@@ -2110,8 +2390,11 @@
       <c r="F50" s="11"/>
       <c r="I50" s="11"/>
       <c r="J50" s="11"/>
-    </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="M50" s="15" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="51" spans="1:13" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A51" s="10"/>
       <c r="B51" s="11"/>
       <c r="C51" s="11"/>
@@ -2119,8 +2402,11 @@
       <c r="F51" s="11"/>
       <c r="I51" s="11"/>
       <c r="J51" s="11"/>
-    </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="M51" s="16" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="52" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A52" s="10"/>
       <c r="B52" s="11"/>
       <c r="C52" s="11"/>
@@ -2129,7 +2415,7 @@
       <c r="I52" s="11"/>
       <c r="J52" s="11"/>
     </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A53" s="10"/>
       <c r="B53" s="11"/>
       <c r="C53" s="11"/>
@@ -2138,7 +2424,7 @@
       <c r="I53" s="11"/>
       <c r="J53" s="11"/>
     </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A54" s="10"/>
       <c r="B54" s="11"/>
       <c r="C54" s="11"/>
@@ -2148,7 +2434,7 @@
       <c r="I54" s="11"/>
       <c r="J54" s="11"/>
     </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A55" s="10"/>
       <c r="B55" s="11"/>
       <c r="C55" s="11"/>
@@ -2157,7 +2443,7 @@
       <c r="I55" s="11"/>
       <c r="J55" s="11"/>
     </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A56" s="10"/>
       <c r="B56" s="11"/>
       <c r="C56" s="11"/>
@@ -2166,7 +2452,7 @@
       <c r="I56" s="11"/>
       <c r="J56" s="11"/>
     </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A57" s="10"/>
       <c r="B57" s="11"/>
       <c r="C57" s="11"/>
@@ -2175,7 +2461,7 @@
       <c r="I57" s="11"/>
       <c r="J57" s="11"/>
     </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A58" s="10"/>
       <c r="B58" s="11"/>
       <c r="C58" s="11"/>
@@ -2184,7 +2470,7 @@
       <c r="I58" s="11"/>
       <c r="J58" s="11"/>
     </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A59" s="10"/>
       <c r="B59" s="11"/>
       <c r="C59" s="11"/>
@@ -2193,7 +2479,7 @@
       <c r="I59" s="11"/>
       <c r="J59" s="11"/>
     </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A60" s="10"/>
       <c r="B60" s="11"/>
       <c r="C60" s="11"/>
@@ -2202,7 +2488,7 @@
       <c r="I60" s="11"/>
       <c r="J60" s="11"/>
     </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A61" s="10"/>
       <c r="B61" s="11"/>
       <c r="C61" s="11"/>
@@ -2211,7 +2497,7 @@
       <c r="I61" s="11"/>
       <c r="J61" s="11"/>
     </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A62" s="10"/>
       <c r="B62" s="11"/>
       <c r="C62" s="11"/>
@@ -2220,7 +2506,7 @@
       <c r="I62" s="11"/>
       <c r="J62" s="11"/>
     </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A63" s="10"/>
       <c r="B63" s="11"/>
       <c r="C63" s="11"/>
@@ -2229,7 +2515,7 @@
       <c r="I63" s="11"/>
       <c r="J63" s="11"/>
     </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A64" s="10"/>
       <c r="B64" s="11"/>
       <c r="C64" s="11"/>
@@ -2238,7 +2524,7 @@
       <c r="I64" s="11"/>
       <c r="J64" s="11"/>
     </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A65" s="10"/>
       <c r="B65" s="11"/>
       <c r="C65" s="11"/>
@@ -2247,7 +2533,7 @@
       <c r="I65" s="11"/>
       <c r="J65" s="11"/>
     </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A66" s="10"/>
       <c r="B66" s="11"/>
       <c r="C66" s="11"/>
@@ -2256,7 +2542,7 @@
       <c r="I66" s="11"/>
       <c r="J66" s="11"/>
     </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A67" s="10"/>
       <c r="B67" s="11"/>
       <c r="C67" s="11"/>
@@ -2265,7 +2551,7 @@
       <c r="I67" s="11"/>
       <c r="J67" s="11"/>
     </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A68" s="10"/>
       <c r="B68" s="11"/>
       <c r="C68" s="11"/>
@@ -2274,7 +2560,7 @@
       <c r="I68" s="11"/>
       <c r="J68" s="11"/>
     </row>
-    <row r="69" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A69" s="10"/>
       <c r="B69" s="11"/>
       <c r="C69" s="11"/>
@@ -2283,142 +2569,142 @@
       <c r="I69" s="11"/>
       <c r="J69" s="11"/>
     </row>
-    <row r="87" spans="4:4" x14ac:dyDescent="0.3">
+    <row r="87" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D87" s="3"/>
     </row>
-    <row r="97" spans="4:4" x14ac:dyDescent="0.3">
+    <row r="97" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D97" s="5"/>
     </row>
-    <row r="130" spans="4:4" x14ac:dyDescent="0.3">
+    <row r="130" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D130" s="3"/>
     </row>
-    <row r="140" spans="4:4" x14ac:dyDescent="0.3">
+    <row r="140" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D140" s="5"/>
     </row>
-    <row r="173" spans="4:4" x14ac:dyDescent="0.3">
+    <row r="173" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D173" s="3"/>
     </row>
-    <row r="183" spans="4:4" x14ac:dyDescent="0.3">
+    <row r="183" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D183" s="5"/>
     </row>
-    <row r="216" spans="4:4" x14ac:dyDescent="0.3">
+    <row r="216" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D216" s="3"/>
     </row>
-    <row r="226" spans="4:4" x14ac:dyDescent="0.3">
+    <row r="226" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D226" s="5"/>
     </row>
-    <row r="259" spans="4:4" x14ac:dyDescent="0.3">
+    <row r="259" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D259" s="3"/>
     </row>
-    <row r="269" spans="4:4" x14ac:dyDescent="0.3">
+    <row r="269" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D269" s="5"/>
     </row>
-    <row r="302" spans="4:4" x14ac:dyDescent="0.3">
+    <row r="302" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D302" s="3"/>
     </row>
-    <row r="312" spans="4:4" x14ac:dyDescent="0.3">
+    <row r="312" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D312" s="5"/>
     </row>
-    <row r="345" spans="4:4" x14ac:dyDescent="0.3">
+    <row r="345" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D345" s="3"/>
     </row>
-    <row r="355" spans="4:4" x14ac:dyDescent="0.3">
+    <row r="355" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D355" s="5"/>
     </row>
-    <row r="388" spans="4:4" x14ac:dyDescent="0.3">
+    <row r="388" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D388" s="3"/>
     </row>
-    <row r="398" spans="4:4" x14ac:dyDescent="0.3">
+    <row r="398" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D398" s="5"/>
     </row>
-    <row r="431" spans="4:4" x14ac:dyDescent="0.3">
+    <row r="431" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D431" s="3"/>
     </row>
-    <row r="441" spans="4:4" x14ac:dyDescent="0.3">
+    <row r="441" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D441" s="5"/>
     </row>
-    <row r="474" spans="4:4" x14ac:dyDescent="0.3">
+    <row r="474" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D474" s="3"/>
     </row>
-    <row r="484" spans="4:4" x14ac:dyDescent="0.3">
+    <row r="484" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D484" s="5"/>
     </row>
-    <row r="517" spans="4:4" x14ac:dyDescent="0.3">
+    <row r="517" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D517" s="3"/>
     </row>
-    <row r="527" spans="4:4" x14ac:dyDescent="0.3">
+    <row r="527" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D527" s="5"/>
     </row>
-    <row r="560" spans="4:4" x14ac:dyDescent="0.3">
+    <row r="560" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D560" s="3"/>
     </row>
-    <row r="570" spans="4:4" x14ac:dyDescent="0.3">
+    <row r="570" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D570" s="5"/>
     </row>
-    <row r="603" spans="4:4" x14ac:dyDescent="0.3">
+    <row r="603" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D603" s="3"/>
     </row>
-    <row r="613" spans="4:4" x14ac:dyDescent="0.3">
+    <row r="613" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D613" s="5"/>
     </row>
-    <row r="646" spans="4:4" x14ac:dyDescent="0.3">
+    <row r="646" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D646" s="3"/>
     </row>
-    <row r="656" spans="4:4" x14ac:dyDescent="0.3">
+    <row r="656" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D656" s="5"/>
     </row>
-    <row r="689" spans="4:4" x14ac:dyDescent="0.3">
+    <row r="689" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D689" s="3"/>
     </row>
-    <row r="699" spans="4:4" x14ac:dyDescent="0.3">
+    <row r="699" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D699" s="5"/>
     </row>
-    <row r="732" spans="4:4" x14ac:dyDescent="0.3">
+    <row r="732" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D732" s="3"/>
     </row>
-    <row r="742" spans="4:4" x14ac:dyDescent="0.3">
+    <row r="742" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D742" s="5"/>
     </row>
-    <row r="775" spans="4:4" x14ac:dyDescent="0.3">
+    <row r="775" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D775" s="3"/>
     </row>
-    <row r="785" spans="4:4" x14ac:dyDescent="0.3">
+    <row r="785" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D785" s="5"/>
     </row>
-    <row r="818" spans="4:4" x14ac:dyDescent="0.3">
+    <row r="818" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D818" s="3"/>
     </row>
-    <row r="828" spans="4:4" x14ac:dyDescent="0.3">
+    <row r="828" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D828" s="5"/>
     </row>
-    <row r="861" spans="4:4" x14ac:dyDescent="0.3">
+    <row r="861" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D861" s="3"/>
     </row>
-    <row r="871" spans="4:4" x14ac:dyDescent="0.3">
+    <row r="871" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D871" s="5"/>
     </row>
-    <row r="904" spans="4:4" x14ac:dyDescent="0.3">
+    <row r="904" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D904" s="3"/>
     </row>
-    <row r="914" spans="4:4" x14ac:dyDescent="0.3">
+    <row r="914" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D914" s="5"/>
     </row>
-    <row r="947" spans="4:4" x14ac:dyDescent="0.3">
+    <row r="947" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D947" s="3"/>
     </row>
-    <row r="957" spans="4:4" x14ac:dyDescent="0.3">
+    <row r="957" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D957" s="5"/>
     </row>
-    <row r="990" spans="4:4" x14ac:dyDescent="0.3">
+    <row r="990" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D990" s="3"/>
     </row>
-    <row r="1000" spans="4:4" x14ac:dyDescent="0.3">
+    <row r="1000" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D1000" s="5"/>
     </row>
-    <row r="1033" spans="4:4" x14ac:dyDescent="0.3">
+    <row r="1033" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D1033" s="3"/>
     </row>
-    <row r="1043" spans="4:4" x14ac:dyDescent="0.3">
+    <row r="1043" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D1043" s="5"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update one marker label of DB3
</commit_message>
<xml_diff>
--- a/data/translation_table.xlsx
+++ b/data/translation_table.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\perla\Documents\AT\TeamProject\GitHub\TeamProject\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3761BDE-A176-4DC2-9104-60950F8CB142}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E246BF3-3571-4C78-ABDA-3F3A9BF53FB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="13728" yWindow="0" windowWidth="9408" windowHeight="12336" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="379" uniqueCount="254">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="379" uniqueCount="252">
   <si>
     <t>Rajagopal2015_ViconPlugInGait.osim</t>
   </si>
@@ -657,16 +657,10 @@
     <t>LFRA</t>
   </si>
   <si>
-    <t>LIAS</t>
-  </si>
-  <si>
     <t>SACR2</t>
   </si>
   <si>
     <t>RFRA</t>
-  </si>
-  <si>
-    <t>RIAS</t>
   </si>
   <si>
     <t>SACR3</t>
@@ -1239,10 +1233,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="H1" t="s">
         <v>6</v>
@@ -1251,13 +1245,13 @@
         <v>7</v>
       </c>
       <c r="J1" s="18" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="M1" s="3" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="N1" s="3" t="s">
         <v>3</v>
@@ -1383,7 +1377,7 @@
         <v>22</v>
       </c>
       <c r="J6" s="19" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="L6" s="1" t="s">
         <v>22</v>
@@ -1453,7 +1447,7 @@
         <v>29</v>
       </c>
       <c r="J9" s="19" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="L9" s="1" t="s">
         <v>29</v>
@@ -1534,7 +1528,7 @@
         <v>40</v>
       </c>
       <c r="J12" s="19" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="L12" s="1" t="s">
         <v>40</v>
@@ -1710,8 +1704,8 @@
       <c r="C19" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="D19" s="16" t="s">
-        <v>210</v>
+      <c r="D19" s="1" t="s">
+        <v>69</v>
       </c>
       <c r="H19" t="s">
         <v>74</v>
@@ -1720,7 +1714,7 @@
         <v>74</v>
       </c>
       <c r="J19" s="19" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="L19" s="1" t="s">
         <v>69</v>
@@ -1749,13 +1743,13 @@
         <v>77</v>
       </c>
       <c r="D20" s="16" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="H20" t="s">
         <v>80</v>
       </c>
       <c r="J20" s="19" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="L20" s="1" t="s">
         <v>75</v>
@@ -1784,7 +1778,7 @@
         <v>83</v>
       </c>
       <c r="D21" s="16" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="I21" t="s">
         <v>86</v>
@@ -1826,7 +1820,7 @@
         <v>93</v>
       </c>
       <c r="J22" s="19" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="L22" s="1" t="s">
         <v>87</v>
@@ -1855,7 +1849,7 @@
         <v>96</v>
       </c>
       <c r="D23" s="16" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="I23" t="s">
         <v>99</v>
@@ -1897,7 +1891,7 @@
         <v>106</v>
       </c>
       <c r="J24" s="19" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="L24" s="1" t="s">
         <v>100</v>
@@ -1935,7 +1929,7 @@
         <v>112</v>
       </c>
       <c r="J25" s="19" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="L25" s="1" t="s">
         <v>107</v>
@@ -1965,7 +1959,7 @@
         <v>113</v>
       </c>
       <c r="J26" s="19" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="L26" s="1" t="s">
         <v>113</v>
@@ -2001,7 +1995,7 @@
         <v>122</v>
       </c>
       <c r="J27" s="19" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="M27" s="1" t="s">
         <v>120</v>
@@ -2028,7 +2022,7 @@
         <v>124</v>
       </c>
       <c r="J28" s="19" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="L28" s="1" t="s">
         <v>124</v>
@@ -2102,7 +2096,7 @@
       </c>
       <c r="C31" s="1"/>
       <c r="D31" s="16" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="J31" s="19"/>
       <c r="M31" s="1" t="s">
@@ -2204,8 +2198,8 @@
       <c r="C35" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="D35" s="16" t="s">
-        <v>213</v>
+      <c r="D35" s="1" t="s">
+        <v>153</v>
       </c>
       <c r="H35" t="s">
         <v>158</v>
@@ -2214,7 +2208,7 @@
         <v>158</v>
       </c>
       <c r="J35" s="19" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="L35" s="1" t="s">
         <v>153</v>
@@ -2243,13 +2237,13 @@
         <v>161</v>
       </c>
       <c r="D36" s="16" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="H36" t="s">
         <v>164</v>
       </c>
       <c r="J36" s="19" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="L36" s="1" t="s">
         <v>159</v>
@@ -2278,7 +2272,7 @@
         <v>167</v>
       </c>
       <c r="D37" s="16" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="I37" t="s">
         <v>169</v>
@@ -2316,7 +2310,7 @@
         <v>176</v>
       </c>
       <c r="J38" s="19" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="L38" s="1" t="s">
         <v>170</v>
@@ -2345,7 +2339,7 @@
         <v>179</v>
       </c>
       <c r="D39" s="16" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="I39" t="s">
         <v>182</v>
@@ -2387,7 +2381,7 @@
         <v>189</v>
       </c>
       <c r="J40" s="19" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="L40" s="1" t="s">
         <v>183</v>
@@ -2425,7 +2419,7 @@
         <v>195</v>
       </c>
       <c r="J41" s="19" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="L41" s="1" t="s">
         <v>190</v>
@@ -2455,7 +2449,7 @@
         <v>196</v>
       </c>
       <c r="J42" s="19" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="L42" s="1" t="s">
         <v>196</v>
@@ -2491,7 +2485,7 @@
         <v>207</v>
       </c>
       <c r="J43" s="19" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="M43" s="1" t="s">
         <v>203</v>
@@ -2519,7 +2513,7 @@
       <c r="B45" s="11"/>
       <c r="C45" s="11"/>
       <c r="D45" s="12" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="M45" s="11"/>
       <c r="N45" s="11"/>
@@ -2531,7 +2525,7 @@
       <c r="B46" s="11"/>
       <c r="C46" s="11"/>
       <c r="D46" s="13" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="M46" s="11"/>
       <c r="N46" s="11"/>
@@ -2543,7 +2537,7 @@
       <c r="B47" s="11"/>
       <c r="C47" s="11"/>
       <c r="D47" s="13" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="M47" s="11"/>
       <c r="N47" s="11"/>
@@ -2555,7 +2549,7 @@
       <c r="B48" s="11"/>
       <c r="C48" s="11"/>
       <c r="D48" s="13" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="M48" s="11"/>
       <c r="N48" s="11"/>
@@ -2567,7 +2561,7 @@
       <c r="B49" s="11"/>
       <c r="C49" s="11"/>
       <c r="D49" s="13" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="M49" s="11"/>
       <c r="N49" s="11"/>
@@ -2579,7 +2573,7 @@
       <c r="B50" s="11"/>
       <c r="C50" s="11"/>
       <c r="D50" s="13" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="M50" s="11"/>
       <c r="N50" s="11"/>
@@ -2591,7 +2585,7 @@
       <c r="B51" s="11"/>
       <c r="C51" s="11"/>
       <c r="D51" s="13" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="M51" s="11"/>
       <c r="N51" s="11"/>
@@ -2603,7 +2597,7 @@
       <c r="B52" s="11"/>
       <c r="C52" s="11"/>
       <c r="D52" s="14" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="M52" s="11"/>
       <c r="N52" s="11"/>
@@ -2615,7 +2609,7 @@
       <c r="B53" s="11"/>
       <c r="C53" s="11"/>
       <c r="D53" s="16" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="M53" s="11"/>
       <c r="N53" s="11"/>
@@ -2627,7 +2621,7 @@
       <c r="B54" s="11"/>
       <c r="C54" s="11"/>
       <c r="D54" s="16" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="L54" s="5"/>
       <c r="M54" s="11"/>
@@ -2640,7 +2634,7 @@
       <c r="B55" s="11"/>
       <c r="C55" s="11"/>
       <c r="D55" s="16" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="M55" s="11"/>
       <c r="N55" s="11"/>
@@ -2652,7 +2646,7 @@
       <c r="B56" s="11"/>
       <c r="C56" s="11"/>
       <c r="D56" s="16" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="M56" s="11"/>
       <c r="N56" s="11"/>

</xml_diff>

<commit_message>
Update translation_table with markers of new DB4_Horst
</commit_message>
<xml_diff>
--- a/data/translation_table.xlsx
+++ b/data/translation_table.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\perla\Documents\AT\TeamProject\GitHub\TeamProject\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E246BF3-3571-4C78-ABDA-3F3A9BF53FB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4716CA56-E1A3-4F88-AC01-8862032C3E44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13728" yWindow="0" windowWidth="9408" windowHeight="12336" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0" iterateDelta="1E-4"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="379" uniqueCount="252">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="417" uniqueCount="285">
   <si>
     <t>Rajagopal2015_ViconPlugInGait.osim</t>
   </si>
@@ -756,9 +757,6 @@
     <t>DB3_Simonlehner</t>
   </si>
   <si>
-    <t>DB4</t>
-  </si>
-  <si>
     <t>LT1</t>
   </si>
   <si>
@@ -781,13 +779,115 @@
   </si>
   <si>
     <t>RS1</t>
+  </si>
+  <si>
+    <t>LLK</t>
+  </si>
+  <si>
+    <t>LLA</t>
+  </si>
+  <si>
+    <t>RLK</t>
+  </si>
+  <si>
+    <t>RLA</t>
+  </si>
+  <si>
+    <t>RFM5</t>
+  </si>
+  <si>
+    <t>LFM5</t>
+  </si>
+  <si>
+    <t>RFM2</t>
+  </si>
+  <si>
+    <t>LFM2</t>
+  </si>
+  <si>
+    <t>DB_Moreira</t>
+  </si>
+  <si>
+    <t>R HEAD</t>
+  </si>
+  <si>
+    <t>L HEAD</t>
+  </si>
+  <si>
+    <t>STERNUM</t>
+  </si>
+  <si>
+    <t>L ACROMION</t>
+  </si>
+  <si>
+    <t>R ACROMION</t>
+  </si>
+  <si>
+    <t>R ILIAC</t>
+  </si>
+  <si>
+    <t>L ILIAC</t>
+  </si>
+  <si>
+    <t>R KNEE LAT</t>
+  </si>
+  <si>
+    <t>L KNEE LAT</t>
+  </si>
+  <si>
+    <t>L ANKLE LAT</t>
+  </si>
+  <si>
+    <t>R ANKLE LAT</t>
+  </si>
+  <si>
+    <t>R HEEL</t>
+  </si>
+  <si>
+    <t>L HEEL</t>
+  </si>
+  <si>
+    <t>R FOOT LAT</t>
+  </si>
+  <si>
+    <t>L FOOT LAT</t>
+  </si>
+  <si>
+    <t>L ELBOW MED</t>
+  </si>
+  <si>
+    <t>R ELBOW MED</t>
+  </si>
+  <si>
+    <t>L WRIST LAT</t>
+  </si>
+  <si>
+    <t>L WIRST MED</t>
+  </si>
+  <si>
+    <t>L HAND</t>
+  </si>
+  <si>
+    <t>R HAND</t>
+  </si>
+  <si>
+    <t>SACRUM</t>
+  </si>
+  <si>
+    <t>R WIRST LAT</t>
+  </si>
+  <si>
+    <t>R WRITS MED</t>
+  </si>
+  <si>
+    <t>DB4_Horst</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -835,6 +935,12 @@
       <color theme="1"/>
       <name val="Aptos Narrow"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -856,7 +962,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -963,11 +1069,31 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="0" tint="-0.499984740745262"/>
+      </left>
+      <right style="thin">
+        <color theme="0" tint="-0.499984740745262"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0" tint="-0.499984740745262"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -981,9 +1107,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1014,6 +1137,28 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1207,11 +1352,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P1043"/>
+  <dimension ref="A1:Q1043"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="3" width="15.77734375" customWidth="1"/>
     <col min="4" max="4" width="17.5546875" customWidth="1"/>
+    <col min="5" max="5" width="17.77734375" customWidth="1"/>
     <col min="8" max="8" width="12.6640625" customWidth="1"/>
     <col min="9" max="9" width="13.44140625" customWidth="1"/>
     <col min="10" max="10" width="16.109375" customWidth="1"/>
@@ -1222,7 +1368,7 @@
     <col min="16" max="16" width="8.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="40.200000000000003" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17" ht="40.200000000000003" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1235,8 +1381,8 @@
       <c r="D1" s="3" t="s">
         <v>242</v>
       </c>
-      <c r="E1" s="3" t="s">
-        <v>243</v>
+      <c r="E1" s="22" t="s">
+        <v>284</v>
       </c>
       <c r="H1" t="s">
         <v>6</v>
@@ -1244,7 +1390,7 @@
       <c r="I1" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="18" t="s">
+      <c r="J1" s="17" t="s">
         <v>221</v>
       </c>
       <c r="L1" s="3" t="s">
@@ -1262,20 +1408,26 @@
       <c r="P1" s="3" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q1" s="22" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>8</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
-      <c r="D2" s="15" t="s">
+      <c r="D2" s="14" t="s">
         <v>8</v>
+      </c>
+      <c r="E2" s="24" t="s">
+        <v>260</v>
       </c>
       <c r="H2" t="s">
         <v>11</v>
       </c>
-      <c r="J2" s="19"/>
+      <c r="J2" s="18"/>
       <c r="L2" s="1" t="s">
         <v>8</v>
       </c>
@@ -1290,19 +1442,22 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
-      <c r="D3" s="15" t="s">
+      <c r="D3" s="14" t="s">
         <v>12</v>
+      </c>
+      <c r="E3" s="24" t="s">
+        <v>261</v>
       </c>
       <c r="H3" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="J3" s="19"/>
+      <c r="J3" s="18"/>
       <c r="L3" s="1" t="s">
         <v>12</v>
       </c>
@@ -1317,16 +1472,16 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
-      <c r="D4" s="15" t="s">
+      <c r="D4" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="J4" s="19"/>
+      <c r="J4" s="18"/>
       <c r="L4" s="1" t="s">
         <v>16</v>
       </c>
@@ -1341,16 +1496,16 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>19</v>
       </c>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
-      <c r="D5" s="15" t="s">
+      <c r="D5" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="J5" s="19"/>
+      <c r="J5" s="18"/>
       <c r="L5" s="1" t="s">
         <v>19</v>
       </c>
@@ -1365,7 +1520,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>22</v>
       </c>
@@ -1373,10 +1528,13 @@
         <v>23</v>
       </c>
       <c r="C6" s="1"/>
-      <c r="D6" s="15" t="s">
+      <c r="D6" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="J6" s="19" t="s">
+      <c r="E6" s="24" t="s">
+        <v>22</v>
+      </c>
+      <c r="J6" s="18" t="s">
         <v>222</v>
       </c>
       <c r="L6" s="1" t="s">
@@ -1393,7 +1551,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>26</v>
       </c>
@@ -1401,10 +1559,10 @@
         <v>27</v>
       </c>
       <c r="C7" s="1"/>
-      <c r="D7" s="15" t="s">
+      <c r="D7" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="J7" s="19"/>
+      <c r="J7" s="18"/>
       <c r="L7" s="1" t="s">
         <v>26</v>
       </c>
@@ -1415,16 +1573,16 @@
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A8" s="1" t="s">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A8" s="19" t="s">
         <v>28</v>
       </c>
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
-      <c r="D8" s="15" t="s">
+      <c r="D8" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="J8" s="19"/>
+      <c r="J8" s="18"/>
       <c r="L8" s="1" t="s">
         <v>28</v>
       </c>
@@ -1435,18 +1593,18 @@
         <v>28</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A9" s="1" t="s">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A9" s="19" t="s">
         <v>29</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C9" s="1"/>
-      <c r="D9" s="15" t="s">
+      <c r="D9" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="J9" s="19" t="s">
+      <c r="J9" s="18" t="s">
         <v>223</v>
       </c>
       <c r="L9" s="1" t="s">
@@ -1463,18 +1621,21 @@
         <v>29</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A10" s="1" t="s">
+    <row r="10" spans="1:17" ht="27" x14ac:dyDescent="0.3">
+      <c r="A10" s="19" t="s">
         <v>33</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>34</v>
       </c>
       <c r="C10" s="1"/>
-      <c r="D10" s="15" t="s">
+      <c r="D10" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="J10" s="19"/>
+      <c r="E10" s="24" t="s">
+        <v>262</v>
+      </c>
+      <c r="J10" s="18"/>
       <c r="L10" s="1" t="s">
         <v>33</v>
       </c>
@@ -1489,19 +1650,22 @@
         <v>33</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A11" s="1" t="s">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A11" s="19" t="s">
         <v>37</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="5"/>
-      <c r="D11" s="15" t="s">
+      <c r="D11" s="14" t="s">
         <v>37</v>
+      </c>
+      <c r="E11" t="s">
+        <v>281</v>
       </c>
       <c r="I11" t="s">
         <v>208</v>
       </c>
-      <c r="J11" s="19"/>
+      <c r="J11" s="18"/>
       <c r="L11" s="5" t="s">
         <v>37</v>
       </c>
@@ -1514,8 +1678,8 @@
       <c r="O11" s="5"/>
       <c r="P11" s="5"/>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A12" s="1" t="s">
+    <row r="12" spans="1:17" ht="40.200000000000003" x14ac:dyDescent="0.3">
+      <c r="A12" s="19" t="s">
         <v>40</v>
       </c>
       <c r="B12" s="1" t="s">
@@ -1524,10 +1688,13 @@
       <c r="C12" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="D12" s="15" t="s">
+      <c r="D12" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="J12" s="19" t="s">
+      <c r="E12" s="24" t="s">
+        <v>263</v>
+      </c>
+      <c r="J12" s="18" t="s">
         <v>224</v>
       </c>
       <c r="L12" s="1" t="s">
@@ -1544,18 +1711,18 @@
         <v>40</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A13" s="1" t="s">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A13" s="19" t="s">
         <v>45</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>46</v>
       </c>
       <c r="C13" s="1"/>
-      <c r="D13" s="15" t="s">
+      <c r="D13" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="J13" s="19"/>
+      <c r="J13" s="18"/>
       <c r="M13" s="1" t="s">
         <v>47</v>
       </c>
@@ -1567,18 +1734,21 @@
         <v>45</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A14" s="1" t="s">
+    <row r="14" spans="1:17" ht="40.200000000000003" x14ac:dyDescent="0.3">
+      <c r="A14" s="19" t="s">
         <v>49</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>50</v>
       </c>
       <c r="C14" s="1"/>
-      <c r="D14" s="15" t="s">
+      <c r="D14" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="J14" s="19"/>
+      <c r="E14" s="25" t="s">
+        <v>275</v>
+      </c>
+      <c r="J14" s="18"/>
       <c r="L14" s="1" t="s">
         <v>49</v>
       </c>
@@ -1593,18 +1763,18 @@
         <v>49</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A15" s="1" t="s">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A15" s="19" t="s">
         <v>53</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>54</v>
       </c>
       <c r="C15" s="1"/>
-      <c r="D15" s="16" t="s">
+      <c r="D15" s="15" t="s">
         <v>209</v>
       </c>
-      <c r="J15" s="19"/>
+      <c r="J15" s="18"/>
       <c r="M15" s="1" t="s">
         <v>55</v>
       </c>
@@ -1616,18 +1786,21 @@
         <v>53</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A16" s="1" t="s">
+    <row r="16" spans="1:17" ht="27" x14ac:dyDescent="0.3">
+      <c r="A16" s="19" t="s">
         <v>57</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>58</v>
       </c>
       <c r="C16" s="1"/>
-      <c r="D16" s="15" t="s">
+      <c r="D16" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="J16" s="19"/>
+      <c r="E16" s="25" t="s">
+        <v>277</v>
+      </c>
+      <c r="J16" s="18"/>
       <c r="L16" s="1" t="s">
         <v>57</v>
       </c>
@@ -1642,18 +1815,21 @@
         <v>57</v>
       </c>
     </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A17" s="1" t="s">
+    <row r="17" spans="1:17" ht="27" x14ac:dyDescent="0.3">
+      <c r="A17" s="19" t="s">
         <v>61</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>62</v>
       </c>
       <c r="C17" s="1"/>
-      <c r="D17" s="15" t="s">
+      <c r="D17" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="J17" s="19"/>
+      <c r="E17" s="25" t="s">
+        <v>278</v>
+      </c>
+      <c r="J17" s="18"/>
       <c r="L17" s="1" t="s">
         <v>61</v>
       </c>
@@ -1668,18 +1844,21 @@
         <v>61</v>
       </c>
     </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A18" s="1" t="s">
+    <row r="18" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A18" s="19" t="s">
         <v>65</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>66</v>
       </c>
       <c r="C18" s="1"/>
-      <c r="D18" s="15" t="s">
+      <c r="D18" s="14" t="s">
         <v>65</v>
       </c>
-      <c r="J18" s="19"/>
+      <c r="E18" s="26" t="s">
+        <v>279</v>
+      </c>
+      <c r="J18" s="18"/>
       <c r="L18" s="1" t="s">
         <v>65</v>
       </c>
@@ -1694,8 +1873,8 @@
         <v>65</v>
       </c>
     </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A19" s="1" t="s">
+    <row r="19" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A19" s="19" t="s">
         <v>69</v>
       </c>
       <c r="B19" s="1" t="s">
@@ -1707,13 +1886,16 @@
       <c r="D19" s="1" t="s">
         <v>69</v>
       </c>
+      <c r="E19" s="23" t="s">
+        <v>266</v>
+      </c>
       <c r="H19" t="s">
         <v>74</v>
       </c>
       <c r="I19" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="J19" s="19" t="s">
+      <c r="J19" s="18" t="s">
         <v>225</v>
       </c>
       <c r="L19" s="1" t="s">
@@ -1731,9 +1913,12 @@
       <c r="P19" s="1" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A20" s="7" t="s">
+      <c r="Q19" s="23" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="20" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A20" s="20" t="s">
         <v>75</v>
       </c>
       <c r="B20" s="1" t="s">
@@ -1742,13 +1927,13 @@
       <c r="C20" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="D20" s="16" t="s">
+      <c r="D20" s="15" t="s">
         <v>210</v>
       </c>
       <c r="H20" t="s">
         <v>80</v>
       </c>
-      <c r="J20" s="19" t="s">
+      <c r="J20" s="18" t="s">
         <v>226</v>
       </c>
       <c r="L20" s="1" t="s">
@@ -1766,9 +1951,12 @@
       <c r="P20" s="1" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A21" s="1" t="s">
+      <c r="Q20" s="23" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="21" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A21" s="19" t="s">
         <v>81</v>
       </c>
       <c r="B21" s="1" t="s">
@@ -1777,13 +1965,13 @@
       <c r="C21" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="D21" s="16" t="s">
-        <v>244</v>
+      <c r="D21" s="15" t="s">
+        <v>243</v>
       </c>
       <c r="I21" t="s">
         <v>86</v>
       </c>
-      <c r="J21" s="19"/>
+      <c r="J21" s="18"/>
       <c r="L21" s="1" t="s">
         <v>81</v>
       </c>
@@ -1800,8 +1988,8 @@
         <v>81</v>
       </c>
     </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A22" s="1" t="s">
+    <row r="22" spans="1:17" ht="27" x14ac:dyDescent="0.3">
+      <c r="A22" s="19" t="s">
         <v>87</v>
       </c>
       <c r="B22" s="1" t="s">
@@ -1810,8 +1998,11 @@
       <c r="C22" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="D22" s="15" t="s">
+      <c r="D22" s="14" t="s">
         <v>87</v>
+      </c>
+      <c r="E22" s="23" t="s">
+        <v>268</v>
       </c>
       <c r="H22" t="s">
         <v>92</v>
@@ -1819,7 +2010,7 @@
       <c r="I22" t="s">
         <v>93</v>
       </c>
-      <c r="J22" s="19" t="s">
+      <c r="J22" s="18" t="s">
         <v>227</v>
       </c>
       <c r="L22" s="1" t="s">
@@ -1837,9 +2028,12 @@
       <c r="P22" s="1" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A23" s="8" t="s">
+      <c r="Q22" s="23" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="23" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A23" s="21" t="s">
         <v>94</v>
       </c>
       <c r="B23" s="1" t="s">
@@ -1848,13 +2042,13 @@
       <c r="C23" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="D23" s="16" t="s">
-        <v>247</v>
+      <c r="D23" s="15" t="s">
+        <v>246</v>
       </c>
       <c r="I23" t="s">
         <v>99</v>
       </c>
-      <c r="J23" s="19"/>
+      <c r="J23" s="18"/>
       <c r="L23" s="1" t="s">
         <v>94</v>
       </c>
@@ -1871,8 +2065,8 @@
         <v>94</v>
       </c>
     </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A24" s="1" t="s">
+    <row r="24" spans="1:17" ht="27" x14ac:dyDescent="0.3">
+      <c r="A24" s="19" t="s">
         <v>100</v>
       </c>
       <c r="B24" s="1" t="s">
@@ -1881,8 +2075,11 @@
       <c r="C24" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="D24" s="15" t="s">
+      <c r="D24" s="14" t="s">
         <v>100</v>
+      </c>
+      <c r="E24" s="24" t="s">
+        <v>269</v>
       </c>
       <c r="H24" t="s">
         <v>105</v>
@@ -1890,7 +2087,7 @@
       <c r="I24" t="s">
         <v>106</v>
       </c>
-      <c r="J24" s="19" t="s">
+      <c r="J24" s="18" t="s">
         <v>228</v>
       </c>
       <c r="L24" s="1" t="s">
@@ -1902,15 +2099,18 @@
       <c r="N24" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="O24" s="9" t="s">
+      <c r="O24" s="8" t="s">
         <v>100</v>
       </c>
       <c r="P24" s="1" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A25" s="1" t="s">
+      <c r="Q24" s="24" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="25" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A25" s="19" t="s">
         <v>107</v>
       </c>
       <c r="B25" s="1" t="s">
@@ -1919,8 +2119,11 @@
       <c r="C25" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="D25" s="15" t="s">
+      <c r="D25" s="14" t="s">
         <v>107</v>
+      </c>
+      <c r="E25" s="24" t="s">
+        <v>272</v>
       </c>
       <c r="H25" t="s">
         <v>112</v>
@@ -1928,7 +2131,7 @@
       <c r="I25" t="s">
         <v>112</v>
       </c>
-      <c r="J25" s="19" t="s">
+      <c r="J25" s="18" t="s">
         <v>229</v>
       </c>
       <c r="L25" s="1" t="s">
@@ -1947,18 +2150,18 @@
         <v>107</v>
       </c>
     </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A26" s="1" t="s">
+    <row r="26" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A26" s="19" t="s">
         <v>113</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>114</v>
       </c>
       <c r="C26" s="1"/>
-      <c r="D26" s="15" t="s">
+      <c r="D26" s="14" t="s">
         <v>113</v>
       </c>
-      <c r="J26" s="19" t="s">
+      <c r="J26" s="18" t="s">
         <v>230</v>
       </c>
       <c r="L26" s="1" t="s">
@@ -1976,9 +2179,12 @@
       <c r="P26" s="1" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A27" s="8" t="s">
+      <c r="Q26" s="23" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="27" spans="1:17" ht="27" x14ac:dyDescent="0.3">
+      <c r="A27" s="21" t="s">
         <v>117</v>
       </c>
       <c r="B27" s="1" t="s">
@@ -1987,14 +2193,17 @@
       <c r="C27" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="D27" s="15"/>
+      <c r="D27" s="14"/>
+      <c r="E27" s="10" t="s">
+        <v>274</v>
+      </c>
       <c r="H27" t="s">
         <v>123</v>
       </c>
       <c r="I27" t="s">
         <v>122</v>
       </c>
-      <c r="J27" s="19" t="s">
+      <c r="J27" s="18" t="s">
         <v>231</v>
       </c>
       <c r="M27" s="1" t="s">
@@ -2007,9 +2216,12 @@
         <v>122</v>
       </c>
       <c r="P27" s="1"/>
-    </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A28" s="8" t="s">
+      <c r="Q27" s="23" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="28" spans="1:17" ht="40.200000000000003" x14ac:dyDescent="0.3">
+      <c r="A28" s="21" t="s">
         <v>124</v>
       </c>
       <c r="B28" s="1" t="s">
@@ -2018,10 +2230,13 @@
       <c r="C28" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="D28" s="15" t="s">
+      <c r="D28" s="14" t="s">
         <v>124</v>
       </c>
-      <c r="J28" s="19" t="s">
+      <c r="E28" s="24" t="s">
+        <v>264</v>
+      </c>
+      <c r="J28" s="18" t="s">
         <v>232</v>
       </c>
       <c r="L28" s="1" t="s">
@@ -2038,18 +2253,18 @@
         <v>124</v>
       </c>
     </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A29" s="1" t="s">
+    <row r="29" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A29" s="19" t="s">
         <v>129</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>130</v>
       </c>
       <c r="C29" s="1"/>
-      <c r="D29" s="15" t="s">
+      <c r="D29" s="14" t="s">
         <v>129</v>
       </c>
-      <c r="J29" s="19"/>
+      <c r="J29" s="18"/>
       <c r="M29" s="1" t="s">
         <v>131</v>
       </c>
@@ -2061,18 +2276,21 @@
         <v>129</v>
       </c>
     </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A30" s="1" t="s">
+    <row r="30" spans="1:17" ht="40.200000000000003" x14ac:dyDescent="0.3">
+      <c r="A30" s="19" t="s">
         <v>133</v>
       </c>
       <c r="B30" s="1" t="s">
         <v>134</v>
       </c>
       <c r="C30" s="1"/>
-      <c r="D30" s="15" t="s">
+      <c r="D30" s="14" t="s">
         <v>133</v>
       </c>
-      <c r="J30" s="19"/>
+      <c r="E30" s="26" t="s">
+        <v>276</v>
+      </c>
+      <c r="J30" s="18"/>
       <c r="L30" s="1" t="s">
         <v>133</v>
       </c>
@@ -2087,18 +2305,18 @@
         <v>133</v>
       </c>
     </row>
-    <row r="31" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A31" s="1" t="s">
+    <row r="31" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A31" s="19" t="s">
         <v>137</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>138</v>
       </c>
       <c r="C31" s="1"/>
-      <c r="D31" s="16" t="s">
+      <c r="D31" s="15" t="s">
         <v>211</v>
       </c>
-      <c r="J31" s="19"/>
+      <c r="J31" s="18"/>
       <c r="M31" s="1" t="s">
         <v>139</v>
       </c>
@@ -2110,18 +2328,21 @@
         <v>137</v>
       </c>
     </row>
-    <row r="32" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A32" s="1" t="s">
+    <row r="32" spans="1:17" ht="27" x14ac:dyDescent="0.3">
+      <c r="A32" s="19" t="s">
         <v>141</v>
       </c>
       <c r="B32" s="1" t="s">
         <v>142</v>
       </c>
       <c r="C32" s="1"/>
-      <c r="D32" s="15" t="s">
+      <c r="D32" s="14" t="s">
         <v>141</v>
       </c>
-      <c r="J32" s="19"/>
+      <c r="E32" s="25" t="s">
+        <v>282</v>
+      </c>
+      <c r="J32" s="18"/>
       <c r="L32" s="1" t="s">
         <v>141</v>
       </c>
@@ -2136,18 +2357,21 @@
         <v>141</v>
       </c>
     </row>
-    <row r="33" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A33" s="8" t="s">
+    <row r="33" spans="1:17" ht="27" x14ac:dyDescent="0.3">
+      <c r="A33" s="21" t="s">
         <v>145</v>
       </c>
       <c r="B33" s="1" t="s">
         <v>146</v>
       </c>
       <c r="C33" s="1"/>
-      <c r="D33" s="15" t="s">
+      <c r="D33" s="14" t="s">
         <v>145</v>
       </c>
-      <c r="J33" s="19"/>
+      <c r="E33" s="25" t="s">
+        <v>283</v>
+      </c>
+      <c r="J33" s="18"/>
       <c r="L33" s="1" t="s">
         <v>145</v>
       </c>
@@ -2162,18 +2386,21 @@
         <v>145</v>
       </c>
     </row>
-    <row r="34" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A34" s="8" t="s">
+    <row r="34" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A34" s="21" t="s">
         <v>149</v>
       </c>
       <c r="B34" s="1" t="s">
         <v>150</v>
       </c>
       <c r="C34" s="1"/>
-      <c r="D34" s="15" t="s">
+      <c r="D34" s="14" t="s">
         <v>149</v>
       </c>
-      <c r="J34" s="19"/>
+      <c r="E34" s="26" t="s">
+        <v>280</v>
+      </c>
+      <c r="J34" s="18"/>
       <c r="L34" s="1" t="s">
         <v>149</v>
       </c>
@@ -2188,7 +2415,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="35" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
         <v>153</v>
       </c>
@@ -2201,13 +2428,16 @@
       <c r="D35" s="1" t="s">
         <v>153</v>
       </c>
+      <c r="E35" s="23" t="s">
+        <v>265</v>
+      </c>
       <c r="H35" t="s">
         <v>158</v>
       </c>
       <c r="I35" s="6" t="s">
         <v>158</v>
       </c>
-      <c r="J35" s="19" t="s">
+      <c r="J35" s="18" t="s">
         <v>233</v>
       </c>
       <c r="L35" s="1" t="s">
@@ -2225,9 +2455,12 @@
       <c r="P35" s="1" t="s">
         <v>153</v>
       </c>
-    </row>
-    <row r="36" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A36" s="8" t="s">
+      <c r="Q35" s="23" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="36" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A36" s="7" t="s">
         <v>159</v>
       </c>
       <c r="B36" s="1" t="s">
@@ -2236,13 +2469,13 @@
       <c r="C36" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="D36" s="16" t="s">
+      <c r="D36" s="15" t="s">
         <v>212</v>
       </c>
       <c r="H36" t="s">
         <v>164</v>
       </c>
-      <c r="J36" s="19" t="s">
+      <c r="J36" s="18" t="s">
         <v>234</v>
       </c>
       <c r="L36" s="1" t="s">
@@ -2260,9 +2493,12 @@
       <c r="P36" s="1" t="s">
         <v>159</v>
       </c>
-    </row>
-    <row r="37" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A37" s="8" t="s">
+      <c r="Q36" s="23" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="37" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A37" s="7" t="s">
         <v>165</v>
       </c>
       <c r="B37" s="1" t="s">
@@ -2271,13 +2507,13 @@
       <c r="C37" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="D37" s="16" t="s">
-        <v>250</v>
+      <c r="D37" s="15" t="s">
+        <v>249</v>
       </c>
       <c r="I37" t="s">
         <v>169</v>
       </c>
-      <c r="J37" s="19"/>
+      <c r="J37" s="18"/>
       <c r="L37" s="1" t="s">
         <v>165</v>
       </c>
@@ -2290,8 +2526,8 @@
         <v>165</v>
       </c>
     </row>
-    <row r="38" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A38" s="8" t="s">
+    <row r="38" spans="1:17" ht="27" x14ac:dyDescent="0.3">
+      <c r="A38" s="7" t="s">
         <v>170</v>
       </c>
       <c r="B38" s="1" t="s">
@@ -2300,8 +2536,11 @@
       <c r="C38" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="D38" s="15" t="s">
+      <c r="D38" s="14" t="s">
         <v>170</v>
+      </c>
+      <c r="E38" s="23" t="s">
+        <v>267</v>
       </c>
       <c r="H38" t="s">
         <v>175</v>
@@ -2309,7 +2548,7 @@
       <c r="I38" t="s">
         <v>176</v>
       </c>
-      <c r="J38" s="19" t="s">
+      <c r="J38" s="18" t="s">
         <v>235</v>
       </c>
       <c r="L38" s="1" t="s">
@@ -2327,9 +2566,12 @@
       <c r="P38" s="1" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="39" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A39" s="8" t="s">
+      <c r="Q38" s="23" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="39" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A39" s="7" t="s">
         <v>177</v>
       </c>
       <c r="B39" s="1" t="s">
@@ -2338,13 +2580,13 @@
       <c r="C39" s="1" t="s">
         <v>179</v>
       </c>
-      <c r="D39" s="16" t="s">
-        <v>251</v>
+      <c r="D39" s="15" t="s">
+        <v>250</v>
       </c>
       <c r="I39" t="s">
         <v>182</v>
       </c>
-      <c r="J39" s="19"/>
+      <c r="J39" s="18"/>
       <c r="L39" s="1" t="s">
         <v>177</v>
       </c>
@@ -2361,7 +2603,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="40" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:17" ht="27" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
         <v>183</v>
       </c>
@@ -2371,8 +2613,11 @@
       <c r="C40" s="1" t="s">
         <v>185</v>
       </c>
-      <c r="D40" s="15" t="s">
+      <c r="D40" s="14" t="s">
         <v>183</v>
+      </c>
+      <c r="E40" s="24" t="s">
+        <v>270</v>
       </c>
       <c r="H40" t="s">
         <v>188</v>
@@ -2380,7 +2625,7 @@
       <c r="I40" t="s">
         <v>189</v>
       </c>
-      <c r="J40" s="19" t="s">
+      <c r="J40" s="18" t="s">
         <v>236</v>
       </c>
       <c r="L40" s="1" t="s">
@@ -2398,8 +2643,11 @@
       <c r="P40" s="1" t="s">
         <v>183</v>
       </c>
-    </row>
-    <row r="41" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q40" s="24" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="41" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
         <v>190</v>
       </c>
@@ -2409,8 +2657,11 @@
       <c r="C41" s="1" t="s">
         <v>192</v>
       </c>
-      <c r="D41" s="15" t="s">
+      <c r="D41" s="14" t="s">
         <v>190</v>
+      </c>
+      <c r="E41" s="24" t="s">
+        <v>271</v>
       </c>
       <c r="H41" t="s">
         <v>195</v>
@@ -2418,7 +2669,7 @@
       <c r="I41" t="s">
         <v>195</v>
       </c>
-      <c r="J41" s="19" t="s">
+      <c r="J41" s="18" t="s">
         <v>237</v>
       </c>
       <c r="L41" s="1" t="s">
@@ -2437,18 +2688,18 @@
         <v>190</v>
       </c>
     </row>
-    <row r="42" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A42" s="8" t="s">
+    <row r="42" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A42" s="7" t="s">
         <v>196</v>
       </c>
       <c r="B42" s="1" t="s">
         <v>197</v>
       </c>
       <c r="C42" s="1"/>
-      <c r="D42" s="15" t="s">
+      <c r="D42" s="14" t="s">
         <v>196</v>
       </c>
-      <c r="J42" s="19" t="s">
+      <c r="J42" s="18" t="s">
         <v>238</v>
       </c>
       <c r="L42" s="1" t="s">
@@ -2466,9 +2717,12 @@
       <c r="P42" s="1" t="s">
         <v>196</v>
       </c>
-    </row>
-    <row r="43" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A43" s="8" t="s">
+      <c r="Q42" s="23" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="43" spans="1:17" ht="27" x14ac:dyDescent="0.3">
+      <c r="A43" s="7" t="s">
         <v>200</v>
       </c>
       <c r="B43" s="1" t="s">
@@ -2477,14 +2731,17 @@
       <c r="C43" s="1" t="s">
         <v>202</v>
       </c>
-      <c r="D43" s="17"/>
+      <c r="D43" s="16"/>
+      <c r="E43" s="10" t="s">
+        <v>273</v>
+      </c>
       <c r="H43" t="s">
         <v>206</v>
       </c>
       <c r="I43" t="s">
         <v>207</v>
       </c>
-      <c r="J43" s="19" t="s">
+      <c r="J43" s="18" t="s">
         <v>239</v>
       </c>
       <c r="M43" s="1" t="s">
@@ -2497,278 +2754,281 @@
         <v>205</v>
       </c>
       <c r="P43" s="1"/>
-    </row>
-    <row r="44" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="10"/>
-      <c r="B44" s="11"/>
-      <c r="C44" s="11"/>
+      <c r="Q43" s="23" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="44" spans="1:17" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A44" s="9"/>
+      <c r="B44" s="10"/>
+      <c r="C44" s="10"/>
       <c r="L44" s="3"/>
-      <c r="M44" s="11"/>
-      <c r="N44" s="11"/>
-      <c r="O44" s="11"/>
-      <c r="P44" s="11"/>
-    </row>
-    <row r="45" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A45" s="10"/>
-      <c r="B45" s="11"/>
-      <c r="C45" s="11"/>
-      <c r="D45" s="12" t="s">
+      <c r="M44" s="10"/>
+      <c r="N44" s="10"/>
+      <c r="O44" s="10"/>
+      <c r="P44" s="10"/>
+    </row>
+    <row r="45" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A45" s="9"/>
+      <c r="B45" s="10"/>
+      <c r="C45" s="10"/>
+      <c r="D45" s="11" t="s">
         <v>220</v>
       </c>
-      <c r="M45" s="11"/>
-      <c r="N45" s="11"/>
-      <c r="O45" s="11"/>
-      <c r="P45" s="11"/>
-    </row>
-    <row r="46" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A46" s="10"/>
-      <c r="B46" s="11"/>
-      <c r="C46" s="11"/>
-      <c r="D46" s="13" t="s">
+      <c r="M45" s="10"/>
+      <c r="N45" s="10"/>
+      <c r="O45" s="10"/>
+      <c r="P45" s="10"/>
+    </row>
+    <row r="46" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A46" s="9"/>
+      <c r="B46" s="10"/>
+      <c r="C46" s="10"/>
+      <c r="D46" s="12" t="s">
         <v>213</v>
       </c>
-      <c r="M46" s="11"/>
-      <c r="N46" s="11"/>
-      <c r="O46" s="11"/>
-      <c r="P46" s="11"/>
-    </row>
-    <row r="47" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A47" s="10"/>
-      <c r="B47" s="11"/>
-      <c r="C47" s="11"/>
-      <c r="D47" s="13" t="s">
+      <c r="M46" s="10"/>
+      <c r="N46" s="10"/>
+      <c r="O46" s="10"/>
+      <c r="P46" s="10"/>
+    </row>
+    <row r="47" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A47" s="9"/>
+      <c r="B47" s="10"/>
+      <c r="C47" s="10"/>
+      <c r="D47" s="12" t="s">
         <v>214</v>
       </c>
-      <c r="M47" s="11"/>
-      <c r="N47" s="11"/>
-      <c r="O47" s="11"/>
-      <c r="P47" s="11"/>
-    </row>
-    <row r="48" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A48" s="10"/>
-      <c r="B48" s="11"/>
-      <c r="C48" s="11"/>
-      <c r="D48" s="13" t="s">
+      <c r="M47" s="10"/>
+      <c r="N47" s="10"/>
+      <c r="O47" s="10"/>
+      <c r="P47" s="10"/>
+    </row>
+    <row r="48" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A48" s="9"/>
+      <c r="B48" s="10"/>
+      <c r="C48" s="10"/>
+      <c r="D48" s="12" t="s">
         <v>215</v>
       </c>
-      <c r="M48" s="11"/>
-      <c r="N48" s="11"/>
-      <c r="O48" s="11"/>
-      <c r="P48" s="11"/>
+      <c r="M48" s="10"/>
+      <c r="N48" s="10"/>
+      <c r="O48" s="10"/>
+      <c r="P48" s="10"/>
     </row>
     <row r="49" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A49" s="10"/>
-      <c r="B49" s="11"/>
-      <c r="C49" s="11"/>
-      <c r="D49" s="13" t="s">
+      <c r="A49" s="9"/>
+      <c r="B49" s="10"/>
+      <c r="C49" s="10"/>
+      <c r="D49" s="12" t="s">
         <v>216</v>
       </c>
-      <c r="M49" s="11"/>
-      <c r="N49" s="11"/>
-      <c r="O49" s="11"/>
-      <c r="P49" s="11"/>
+      <c r="M49" s="10"/>
+      <c r="N49" s="10"/>
+      <c r="O49" s="10"/>
+      <c r="P49" s="10"/>
     </row>
     <row r="50" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A50" s="10"/>
-      <c r="B50" s="11"/>
-      <c r="C50" s="11"/>
-      <c r="D50" s="13" t="s">
+      <c r="A50" s="9"/>
+      <c r="B50" s="10"/>
+      <c r="C50" s="10"/>
+      <c r="D50" s="12" t="s">
         <v>217</v>
       </c>
-      <c r="M50" s="11"/>
-      <c r="N50" s="11"/>
-      <c r="O50" s="11"/>
-      <c r="P50" s="11"/>
+      <c r="M50" s="10"/>
+      <c r="N50" s="10"/>
+      <c r="O50" s="10"/>
+      <c r="P50" s="10"/>
     </row>
     <row r="51" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A51" s="10"/>
-      <c r="B51" s="11"/>
-      <c r="C51" s="11"/>
-      <c r="D51" s="13" t="s">
+      <c r="A51" s="9"/>
+      <c r="B51" s="10"/>
+      <c r="C51" s="10"/>
+      <c r="D51" s="12" t="s">
         <v>218</v>
       </c>
-      <c r="M51" s="11"/>
-      <c r="N51" s="11"/>
-      <c r="O51" s="11"/>
-      <c r="P51" s="11"/>
+      <c r="M51" s="10"/>
+      <c r="N51" s="10"/>
+      <c r="O51" s="10"/>
+      <c r="P51" s="10"/>
     </row>
     <row r="52" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A52" s="10"/>
-      <c r="B52" s="11"/>
-      <c r="C52" s="11"/>
-      <c r="D52" s="14" t="s">
+      <c r="A52" s="9"/>
+      <c r="B52" s="10"/>
+      <c r="C52" s="10"/>
+      <c r="D52" s="13" t="s">
         <v>219</v>
       </c>
-      <c r="M52" s="11"/>
-      <c r="N52" s="11"/>
-      <c r="O52" s="11"/>
-      <c r="P52" s="11"/>
+      <c r="M52" s="10"/>
+      <c r="N52" s="10"/>
+      <c r="O52" s="10"/>
+      <c r="P52" s="10"/>
     </row>
     <row r="53" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A53" s="10"/>
-      <c r="B53" s="11"/>
-      <c r="C53" s="11"/>
-      <c r="D53" s="16" t="s">
+      <c r="A53" s="9"/>
+      <c r="B53" s="10"/>
+      <c r="C53" s="10"/>
+      <c r="D53" s="15" t="s">
+        <v>244</v>
+      </c>
+      <c r="M53" s="10"/>
+      <c r="N53" s="10"/>
+      <c r="O53" s="10"/>
+      <c r="P53" s="10"/>
+    </row>
+    <row r="54" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A54" s="9"/>
+      <c r="B54" s="10"/>
+      <c r="C54" s="10"/>
+      <c r="D54" s="15" t="s">
         <v>245</v>
       </c>
-      <c r="M53" s="11"/>
-      <c r="N53" s="11"/>
-      <c r="O53" s="11"/>
-      <c r="P53" s="11"/>
-    </row>
-    <row r="54" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A54" s="10"/>
-      <c r="B54" s="11"/>
-      <c r="C54" s="11"/>
-      <c r="D54" s="16" t="s">
-        <v>246</v>
-      </c>
       <c r="L54" s="5"/>
-      <c r="M54" s="11"/>
-      <c r="N54" s="11"/>
-      <c r="O54" s="11"/>
-      <c r="P54" s="11"/>
+      <c r="M54" s="10"/>
+      <c r="N54" s="10"/>
+      <c r="O54" s="10"/>
+      <c r="P54" s="10"/>
     </row>
     <row r="55" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A55" s="10"/>
-      <c r="B55" s="11"/>
-      <c r="C55" s="11"/>
-      <c r="D55" s="16" t="s">
+      <c r="A55" s="9"/>
+      <c r="B55" s="10"/>
+      <c r="C55" s="10"/>
+      <c r="D55" s="15" t="s">
+        <v>247</v>
+      </c>
+      <c r="M55" s="10"/>
+      <c r="N55" s="10"/>
+      <c r="O55" s="10"/>
+      <c r="P55" s="10"/>
+    </row>
+    <row r="56" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A56" s="9"/>
+      <c r="B56" s="10"/>
+      <c r="C56" s="10"/>
+      <c r="D56" s="15" t="s">
         <v>248</v>
       </c>
-      <c r="M55" s="11"/>
-      <c r="N55" s="11"/>
-      <c r="O55" s="11"/>
-      <c r="P55" s="11"/>
-    </row>
-    <row r="56" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A56" s="10"/>
-      <c r="B56" s="11"/>
-      <c r="C56" s="11"/>
-      <c r="D56" s="16" t="s">
-        <v>249</v>
-      </c>
-      <c r="M56" s="11"/>
-      <c r="N56" s="11"/>
-      <c r="O56" s="11"/>
-      <c r="P56" s="11"/>
+      <c r="M56" s="10"/>
+      <c r="N56" s="10"/>
+      <c r="O56" s="10"/>
+      <c r="P56" s="10"/>
     </row>
     <row r="57" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A57" s="10"/>
-      <c r="B57" s="11"/>
-      <c r="C57" s="11"/>
-      <c r="M57" s="11"/>
-      <c r="N57" s="11"/>
-      <c r="O57" s="11"/>
-      <c r="P57" s="11"/>
+      <c r="A57" s="9"/>
+      <c r="B57" s="10"/>
+      <c r="C57" s="10"/>
+      <c r="M57" s="10"/>
+      <c r="N57" s="10"/>
+      <c r="O57" s="10"/>
+      <c r="P57" s="10"/>
     </row>
     <row r="58" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A58" s="10"/>
-      <c r="B58" s="11"/>
-      <c r="C58" s="11"/>
-      <c r="M58" s="11"/>
-      <c r="N58" s="11"/>
-      <c r="O58" s="11"/>
-      <c r="P58" s="11"/>
+      <c r="A58" s="9"/>
+      <c r="B58" s="10"/>
+      <c r="C58" s="10"/>
+      <c r="M58" s="10"/>
+      <c r="N58" s="10"/>
+      <c r="O58" s="10"/>
+      <c r="P58" s="10"/>
     </row>
     <row r="59" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A59" s="10"/>
-      <c r="B59" s="11"/>
-      <c r="C59" s="11"/>
-      <c r="M59" s="11"/>
-      <c r="N59" s="11"/>
-      <c r="O59" s="11"/>
-      <c r="P59" s="11"/>
+      <c r="A59" s="9"/>
+      <c r="B59" s="10"/>
+      <c r="C59" s="10"/>
+      <c r="M59" s="10"/>
+      <c r="N59" s="10"/>
+      <c r="O59" s="10"/>
+      <c r="P59" s="10"/>
     </row>
     <row r="60" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A60" s="10"/>
-      <c r="B60" s="11"/>
-      <c r="C60" s="11"/>
-      <c r="M60" s="11"/>
-      <c r="N60" s="11"/>
-      <c r="O60" s="11"/>
-      <c r="P60" s="11"/>
+      <c r="A60" s="9"/>
+      <c r="B60" s="10"/>
+      <c r="C60" s="10"/>
+      <c r="M60" s="10"/>
+      <c r="N60" s="10"/>
+      <c r="O60" s="10"/>
+      <c r="P60" s="10"/>
     </row>
     <row r="61" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A61" s="10"/>
-      <c r="B61" s="11"/>
-      <c r="C61" s="11"/>
-      <c r="M61" s="11"/>
-      <c r="N61" s="11"/>
-      <c r="O61" s="11"/>
-      <c r="P61" s="11"/>
+      <c r="A61" s="9"/>
+      <c r="B61" s="10"/>
+      <c r="C61" s="10"/>
+      <c r="M61" s="10"/>
+      <c r="N61" s="10"/>
+      <c r="O61" s="10"/>
+      <c r="P61" s="10"/>
     </row>
     <row r="62" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A62" s="10"/>
-      <c r="B62" s="11"/>
-      <c r="C62" s="11"/>
-      <c r="M62" s="11"/>
-      <c r="N62" s="11"/>
-      <c r="O62" s="11"/>
-      <c r="P62" s="11"/>
+      <c r="A62" s="9"/>
+      <c r="B62" s="10"/>
+      <c r="C62" s="10"/>
+      <c r="M62" s="10"/>
+      <c r="N62" s="10"/>
+      <c r="O62" s="10"/>
+      <c r="P62" s="10"/>
     </row>
     <row r="63" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A63" s="10"/>
-      <c r="B63" s="11"/>
-      <c r="C63" s="11"/>
-      <c r="M63" s="11"/>
-      <c r="N63" s="11"/>
-      <c r="O63" s="11"/>
-      <c r="P63" s="11"/>
+      <c r="A63" s="9"/>
+      <c r="B63" s="10"/>
+      <c r="C63" s="10"/>
+      <c r="M63" s="10"/>
+      <c r="N63" s="10"/>
+      <c r="O63" s="10"/>
+      <c r="P63" s="10"/>
     </row>
     <row r="64" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A64" s="10"/>
-      <c r="B64" s="11"/>
-      <c r="C64" s="11"/>
-      <c r="M64" s="11"/>
-      <c r="N64" s="11"/>
-      <c r="O64" s="11"/>
-      <c r="P64" s="11"/>
+      <c r="A64" s="9"/>
+      <c r="B64" s="10"/>
+      <c r="C64" s="10"/>
+      <c r="M64" s="10"/>
+      <c r="N64" s="10"/>
+      <c r="O64" s="10"/>
+      <c r="P64" s="10"/>
     </row>
     <row r="65" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A65" s="10"/>
-      <c r="B65" s="11"/>
-      <c r="C65" s="11"/>
-      <c r="M65" s="11"/>
-      <c r="N65" s="11"/>
-      <c r="O65" s="11"/>
-      <c r="P65" s="11"/>
+      <c r="A65" s="9"/>
+      <c r="B65" s="10"/>
+      <c r="C65" s="10"/>
+      <c r="M65" s="10"/>
+      <c r="N65" s="10"/>
+      <c r="O65" s="10"/>
+      <c r="P65" s="10"/>
     </row>
     <row r="66" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A66" s="10"/>
-      <c r="B66" s="11"/>
-      <c r="C66" s="11"/>
-      <c r="M66" s="11"/>
-      <c r="N66" s="11"/>
-      <c r="O66" s="11"/>
-      <c r="P66" s="11"/>
+      <c r="A66" s="9"/>
+      <c r="B66" s="10"/>
+      <c r="C66" s="10"/>
+      <c r="M66" s="10"/>
+      <c r="N66" s="10"/>
+      <c r="O66" s="10"/>
+      <c r="P66" s="10"/>
     </row>
     <row r="67" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A67" s="10"/>
-      <c r="B67" s="11"/>
-      <c r="C67" s="11"/>
-      <c r="M67" s="11"/>
-      <c r="N67" s="11"/>
-      <c r="O67" s="11"/>
-      <c r="P67" s="11"/>
+      <c r="A67" s="9"/>
+      <c r="B67" s="10"/>
+      <c r="C67" s="10"/>
+      <c r="M67" s="10"/>
+      <c r="N67" s="10"/>
+      <c r="O67" s="10"/>
+      <c r="P67" s="10"/>
     </row>
     <row r="68" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A68" s="10"/>
-      <c r="B68" s="11"/>
-      <c r="C68" s="11"/>
-      <c r="M68" s="11"/>
-      <c r="N68" s="11"/>
-      <c r="O68" s="11"/>
-      <c r="P68" s="11"/>
+      <c r="A68" s="9"/>
+      <c r="B68" s="10"/>
+      <c r="C68" s="10"/>
+      <c r="M68" s="10"/>
+      <c r="N68" s="10"/>
+      <c r="O68" s="10"/>
+      <c r="P68" s="10"/>
     </row>
     <row r="69" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A69" s="10"/>
-      <c r="B69" s="11"/>
-      <c r="C69" s="11"/>
-      <c r="M69" s="11"/>
-      <c r="N69" s="11"/>
-      <c r="O69" s="11"/>
-      <c r="P69" s="11"/>
+      <c r="A69" s="9"/>
+      <c r="B69" s="10"/>
+      <c r="C69" s="10"/>
+      <c r="M69" s="10"/>
+      <c r="N69" s="10"/>
+      <c r="O69" s="10"/>
+      <c r="P69" s="10"/>
     </row>
     <row r="87" spans="12:12" x14ac:dyDescent="0.3">
       <c r="L87" s="3"/>

</xml_diff>